<commit_message>
bloc2 : add fiche de specs
</commit_message>
<xml_diff>
--- a/Bloc 2/docs/Besoins du business case.xlsx
+++ b/Bloc 2/docs/Besoins du business case.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ronan.guillou\Documents\Formation_jedha\Certification_RNCP41993\Bloc 2\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383655FD-93FA-4A14-B7D0-13685D29DDB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{893A548E-A250-4B4A-B8A3-59887860F932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{59E4A163-76CB-4141-A26D-230667CF9957}"/>
   </bookViews>
@@ -284,7 +284,7 @@
     <t>Synchone</t>
   </si>
   <si>
-    <t>Sauvegarde, journlisation</t>
+    <t>Sauvegarde, journalisation, multi-zone</t>
   </si>
 </sst>
 </file>
@@ -674,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CFB8B5A-C8CE-4113-A148-E2F4A39DDDE3}">
-  <dimension ref="A5:XFD59"/>
+  <dimension ref="A5:XFD58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="71.7109375" customWidth="1"/>
@@ -722,7 +722,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -730,7 +730,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
@@ -738,12 +738,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>9</v>
       </c>
@@ -49994,7 +49994,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>34</v>
       </c>
@@ -50002,7 +50002,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>35</v>
       </c>
@@ -50010,7 +50010,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>33</v>
       </c>
@@ -50018,7 +50018,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>36</v>
       </c>
@@ -50026,12 +50026,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>42</v>
       </c>
@@ -50039,22 +50039,22 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="44" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>48</v>
       </c>
@@ -50062,7 +50062,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>49</v>
       </c>
@@ -50070,7 +50070,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="46" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>52</v>
       </c>
@@ -50078,7 +50078,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="47" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>54</v>
       </c>
@@ -50086,7 +50086,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="48" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>56</v>
       </c>
@@ -50094,7 +50094,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="49" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>58</v>
       </c>
@@ -50102,7 +50102,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>60</v>
       </c>
@@ -50110,7 +50110,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="51" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>62</v>
       </c>
@@ -50118,7 +50118,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="52" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>67</v>
       </c>
@@ -50126,7 +50126,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="53" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>66</v>
       </c>
@@ -50134,7 +50134,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>65</v>
       </c>
@@ -50142,7 +50142,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="55" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>69</v>
       </c>
@@ -50150,12 +50150,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="56" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="57" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>72</v>
       </c>
@@ -50163,7 +50163,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="58" spans="1:2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>70</v>
       </c>
@@ -50171,7 +50171,6 @@
         <v>73</v>
       </c>
     </row>
-    <row r="59" spans="1:2" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>